<commit_message>
add:  Crud Impuestos Items
</commit_message>
<xml_diff>
--- a/api/src/main/resources/Permisos.xlsx
+++ b/api/src/main/resources/Permisos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF5489F-8B71-4D62-9831-34867D8F6C85}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4871B7E8-F412-48C3-B4D1-5A43A6086B38}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{52F446C3-5058-4B3C-98DD-BC70BC1F7036}"/>
   </bookViews>
@@ -987,18 +987,6 @@
     <t>CRM</t>
   </si>
   <si>
-    <t>CR_CC_CR</t>
-  </si>
-  <si>
-    <t>CR_CC_MO</t>
-  </si>
-  <si>
-    <t>CR_CC_EL</t>
-  </si>
-  <si>
-    <t>CR_CC_VR</t>
-  </si>
-  <si>
     <t>CR_CT_CR</t>
   </si>
   <si>
@@ -1930,6 +1918,18 @@
   </si>
   <si>
     <t>api/v1.0/cxp-pagos/{idEmpresa}/{idGrupoFactura}</t>
+  </si>
+  <si>
+    <t>CF_CC_CR</t>
+  </si>
+  <si>
+    <t>CF_CC_MO</t>
+  </si>
+  <si>
+    <t>CF_CC_EL</t>
+  </si>
+  <si>
+    <t>CF_CC_VR</t>
   </si>
 </sst>
 </file>
@@ -2099,6 +2099,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2106,12 +2112,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2428,7 +2428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0CD9FE9-FD70-4C80-A858-550DB4967E51}">
-  <dimension ref="A1:L357"/>
+  <dimension ref="A1:L362"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" customWidth="1"/>
@@ -2458,12 +2458,12 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -2506,10 +2506,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D4" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>143</v>
@@ -2523,10 +2523,10 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D5" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>143</v>
@@ -2540,10 +2540,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D6" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>143</v>
@@ -2557,10 +2557,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D7" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>145</v>
@@ -2574,10 +2574,10 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D8" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>145</v>
@@ -2591,10 +2591,10 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D9" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>145</v>
@@ -2608,10 +2608,10 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D10" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>143</v>
@@ -2625,10 +2625,10 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D11" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>143</v>
@@ -2642,10 +2642,10 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D12" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>143</v>
@@ -2659,10 +2659,10 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D13" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>143</v>
@@ -2674,7 +2674,7 @@
         <v>144</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2685,10 +2685,10 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D14" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>143</v>
@@ -2700,7 +2700,7 @@
         <v>144</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2711,10 +2711,10 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D15" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>143</v>
@@ -2726,7 +2726,7 @@
         <v>144</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2791,10 +2791,10 @@
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D19" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>151</v>
@@ -2808,10 +2808,10 @@
         <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D20" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>151</v>
@@ -2825,10 +2825,10 @@
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D21" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>151</v>
@@ -2842,10 +2842,10 @@
         <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D22" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>152</v>
@@ -2859,10 +2859,10 @@
         <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D23" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>152</v>
@@ -2876,10 +2876,10 @@
         <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D24" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>152</v>
@@ -2893,10 +2893,10 @@
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D25" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>151</v>
@@ -2910,10 +2910,10 @@
         <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D26" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>151</v>
@@ -2927,10 +2927,10 @@
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D27" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>151</v>
@@ -2944,10 +2944,10 @@
         <v>12</v>
       </c>
       <c r="C28" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D28" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>151</v>
@@ -2964,10 +2964,10 @@
         <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D29" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>151</v>
@@ -2984,10 +2984,10 @@
         <v>12</v>
       </c>
       <c r="C30" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D30" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>151</v>
@@ -3021,10 +3021,10 @@
         <v>13</v>
       </c>
       <c r="C32" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D32" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>154</v>
@@ -3038,10 +3038,10 @@
         <v>13</v>
       </c>
       <c r="C33" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D33" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>154</v>
@@ -3055,10 +3055,10 @@
         <v>13</v>
       </c>
       <c r="C34" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D34" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>154</v>
@@ -3072,10 +3072,10 @@
         <v>13</v>
       </c>
       <c r="C35" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D35" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>155</v>
@@ -3089,10 +3089,10 @@
         <v>13</v>
       </c>
       <c r="C36" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D36" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>155</v>
@@ -3106,10 +3106,10 @@
         <v>13</v>
       </c>
       <c r="C37" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D37" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>155</v>
@@ -3123,10 +3123,10 @@
         <v>13</v>
       </c>
       <c r="C38" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D38" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>154</v>
@@ -3140,10 +3140,10 @@
         <v>13</v>
       </c>
       <c r="C39" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D39" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>154</v>
@@ -3157,10 +3157,10 @@
         <v>13</v>
       </c>
       <c r="C40" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D40" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>154</v>
@@ -3174,10 +3174,10 @@
         <v>13</v>
       </c>
       <c r="C41" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D41" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>154</v>
@@ -3194,10 +3194,10 @@
         <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D42" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>154</v>
@@ -3214,10 +3214,10 @@
         <v>13</v>
       </c>
       <c r="C43" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D43" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>154</v>
@@ -3377,10 +3377,10 @@
         <v>29</v>
       </c>
       <c r="C52" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D52" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>165</v>
@@ -3394,10 +3394,10 @@
         <v>29</v>
       </c>
       <c r="C53" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D53" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>165</v>
@@ -3411,10 +3411,10 @@
         <v>29</v>
       </c>
       <c r="C54" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D54" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>165</v>
@@ -3428,10 +3428,10 @@
         <v>29</v>
       </c>
       <c r="C55" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D55" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>166</v>
@@ -3445,10 +3445,10 @@
         <v>29</v>
       </c>
       <c r="C56" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D56" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>166</v>
@@ -3462,10 +3462,10 @@
         <v>29</v>
       </c>
       <c r="C57" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D57" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="E57" s="4" t="s">
         <v>166</v>
@@ -3479,10 +3479,10 @@
         <v>29</v>
       </c>
       <c r="C58" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D58" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>165</v>
@@ -3496,10 +3496,10 @@
         <v>29</v>
       </c>
       <c r="C59" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D59" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>165</v>
@@ -3513,10 +3513,10 @@
         <v>29</v>
       </c>
       <c r="C60" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D60" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>165</v>
@@ -3530,10 +3530,10 @@
         <v>29</v>
       </c>
       <c r="C61" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D61" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>165</v>
@@ -3553,10 +3553,10 @@
         <v>29</v>
       </c>
       <c r="C62" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D62" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>165</v>
@@ -3576,10 +3576,10 @@
         <v>29</v>
       </c>
       <c r="C63" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D63" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>165</v>
@@ -3637,10 +3637,10 @@
         <v>44</v>
       </c>
       <c r="C66" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D66" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>172</v>
@@ -3655,10 +3655,10 @@
         <v>44</v>
       </c>
       <c r="C67" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D67" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>172</v>
@@ -3673,10 +3673,10 @@
         <v>44</v>
       </c>
       <c r="C68" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D68" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>172</v>
@@ -3690,10 +3690,10 @@
         <v>44</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D69" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>172</v>
@@ -3707,10 +3707,10 @@
         <v>44</v>
       </c>
       <c r="C70" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D70" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>172</v>
@@ -3724,10 +3724,10 @@
         <v>44</v>
       </c>
       <c r="C71" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D71" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>172</v>
@@ -3741,10 +3741,10 @@
         <v>44</v>
       </c>
       <c r="C72" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D72" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>172</v>
@@ -3764,10 +3764,10 @@
         <v>44</v>
       </c>
       <c r="C73" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D73" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>172</v>
@@ -3787,10 +3787,10 @@
         <v>44</v>
       </c>
       <c r="C74" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D74" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>172</v>
@@ -3847,10 +3847,10 @@
         <v>41</v>
       </c>
       <c r="C77" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D77" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>177</v>
@@ -3864,10 +3864,10 @@
         <v>41</v>
       </c>
       <c r="C78" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D78" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>177</v>
@@ -3881,10 +3881,10 @@
         <v>41</v>
       </c>
       <c r="C79" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D79" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>177</v>
@@ -3898,10 +3898,10 @@
         <v>41</v>
       </c>
       <c r="C80" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D80" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>177</v>
@@ -3915,10 +3915,10 @@
         <v>41</v>
       </c>
       <c r="C81" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D81" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>177</v>
@@ -3932,10 +3932,10 @@
         <v>41</v>
       </c>
       <c r="C82" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D82" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E82" s="4" t="s">
         <v>177</v>
@@ -3949,10 +3949,10 @@
         <v>41</v>
       </c>
       <c r="C83" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D83" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="E83" s="4" t="s">
         <v>177</v>
@@ -3969,10 +3969,10 @@
         <v>41</v>
       </c>
       <c r="C84" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D84" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="E84" s="4" t="s">
         <v>177</v>
@@ -3989,10 +3989,10 @@
         <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D85" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="E85" s="4" t="s">
         <v>177</v>
@@ -4120,10 +4120,10 @@
         <v>80</v>
       </c>
       <c r="C92" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D92" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="E92" s="4" t="s">
         <v>189</v>
@@ -4137,10 +4137,10 @@
         <v>80</v>
       </c>
       <c r="C93" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D93" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="E93" s="4" t="s">
         <v>189</v>
@@ -4154,10 +4154,10 @@
         <v>80</v>
       </c>
       <c r="C94" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D94" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="E94" s="4" t="s">
         <v>189</v>
@@ -4171,10 +4171,10 @@
         <v>80</v>
       </c>
       <c r="C95" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D95" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="E95" s="4" t="s">
         <v>189</v>
@@ -4188,10 +4188,10 @@
         <v>80</v>
       </c>
       <c r="C96" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D96" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="E96" s="4" t="s">
         <v>189</v>
@@ -4205,10 +4205,10 @@
         <v>80</v>
       </c>
       <c r="C97" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D97" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="E97" s="4" t="s">
         <v>189</v>
@@ -4222,10 +4222,10 @@
         <v>80</v>
       </c>
       <c r="C98" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D98" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>189</v>
@@ -4245,10 +4245,10 @@
         <v>80</v>
       </c>
       <c r="C99" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D99" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>189</v>
@@ -4268,10 +4268,10 @@
         <v>80</v>
       </c>
       <c r="C100" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D100" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="E100" s="4" t="s">
         <v>189</v>
@@ -4558,10 +4558,10 @@
         <v>32</v>
       </c>
       <c r="C117" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D117" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="E117" s="4" t="s">
         <v>207</v>
@@ -4575,10 +4575,10 @@
         <v>32</v>
       </c>
       <c r="C118" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D118" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="E118" s="4" t="s">
         <v>207</v>
@@ -4592,10 +4592,10 @@
         <v>32</v>
       </c>
       <c r="C119" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D119" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="E119" s="4" t="s">
         <v>207</v>
@@ -4609,10 +4609,10 @@
         <v>32</v>
       </c>
       <c r="C120" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D120" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
@@ -4623,10 +4623,10 @@
         <v>32</v>
       </c>
       <c r="C121" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D121" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="F121" s="4"/>
       <c r="G121" s="4"/>
@@ -4639,10 +4639,10 @@
         <v>32</v>
       </c>
       <c r="C122" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D122" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
@@ -4653,10 +4653,10 @@
         <v>32</v>
       </c>
       <c r="C123" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D123" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="E123" s="4" t="s">
         <v>207</v>
@@ -4670,10 +4670,10 @@
         <v>32</v>
       </c>
       <c r="C124" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D124" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="E124" s="4" t="s">
         <v>207</v>
@@ -4687,10 +4687,10 @@
         <v>32</v>
       </c>
       <c r="C125" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D125" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="E125" s="4" t="s">
         <v>207</v>
@@ -4704,10 +4704,10 @@
         <v>32</v>
       </c>
       <c r="C126" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D126" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="E126" s="4" t="s">
         <v>207</v>
@@ -4727,10 +4727,10 @@
         <v>32</v>
       </c>
       <c r="C127" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D127" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="E127" s="4" t="s">
         <v>207</v>
@@ -4750,10 +4750,10 @@
         <v>32</v>
       </c>
       <c r="C128" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D128" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="E128" s="4" t="s">
         <v>207</v>
@@ -4813,10 +4813,10 @@
         <v>36</v>
       </c>
       <c r="C131" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D131" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="E131" s="4" t="s">
         <v>213</v>
@@ -4834,10 +4834,10 @@
         <v>36</v>
       </c>
       <c r="C132" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D132" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="E132" s="4" t="s">
         <v>213</v>
@@ -4855,10 +4855,10 @@
         <v>36</v>
       </c>
       <c r="C133" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D133" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>213</v>
@@ -4876,10 +4876,10 @@
         <v>36</v>
       </c>
       <c r="C134" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D134" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>214</v>
@@ -4895,10 +4895,10 @@
         <v>36</v>
       </c>
       <c r="C135" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D135" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="E135" s="4" t="s">
         <v>214</v>
@@ -4914,10 +4914,10 @@
         <v>36</v>
       </c>
       <c r="C136" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D136" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="E136" s="4" t="s">
         <v>214</v>
@@ -4933,10 +4933,10 @@
         <v>36</v>
       </c>
       <c r="C137" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D137" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="E137" s="4" t="s">
         <v>214</v>
@@ -4954,10 +4954,10 @@
         <v>36</v>
       </c>
       <c r="C138" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D138" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="E138" s="4" t="s">
         <v>214</v>
@@ -4974,10 +4974,10 @@
         <v>36</v>
       </c>
       <c r="C139" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D139" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="E139" s="4" t="s">
         <v>214</v>
@@ -5032,10 +5032,10 @@
         <v>41</v>
       </c>
       <c r="C142" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D142" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="E142" s="4" t="s">
         <v>234</v>
@@ -5050,10 +5050,10 @@
         <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D143" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="E143" s="4" t="s">
         <v>234</v>
@@ -5068,10 +5068,10 @@
         <v>41</v>
       </c>
       <c r="C144" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D144" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="E144" s="4" t="s">
         <v>234</v>
@@ -5086,10 +5086,10 @@
         <v>41</v>
       </c>
       <c r="C145" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D145" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="E145" s="4" t="s">
         <v>235</v>
@@ -5104,10 +5104,10 @@
         <v>41</v>
       </c>
       <c r="C146" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D146" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="E146" s="4" t="s">
         <v>235</v>
@@ -5121,10 +5121,10 @@
         <v>41</v>
       </c>
       <c r="C147" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D147" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="E147" s="4" t="s">
         <v>235</v>
@@ -5138,10 +5138,10 @@
         <v>41</v>
       </c>
       <c r="C148" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D148" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="E148" s="4" t="s">
         <v>234</v>
@@ -5155,10 +5155,10 @@
         <v>41</v>
       </c>
       <c r="C149" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D149" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="E149" s="4" t="s">
         <v>234</v>
@@ -5172,10 +5172,10 @@
         <v>41</v>
       </c>
       <c r="C150" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D150" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="E150" s="4" t="s">
         <v>234</v>
@@ -5189,10 +5189,10 @@
         <v>41</v>
       </c>
       <c r="C151" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D151" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="E151" s="4" t="s">
         <v>234</v>
@@ -5212,10 +5212,10 @@
         <v>41</v>
       </c>
       <c r="C152" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D152" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="E152" s="4" t="s">
         <v>234</v>
@@ -5235,10 +5235,10 @@
         <v>41</v>
       </c>
       <c r="C153" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D153" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="E153" s="4" t="s">
         <v>234</v>
@@ -5296,10 +5296,10 @@
         <v>49</v>
       </c>
       <c r="C156" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D156" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="E156" s="4" t="s">
         <v>241</v>
@@ -5313,10 +5313,10 @@
         <v>49</v>
       </c>
       <c r="C157" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D157" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="E157" s="4" t="s">
         <v>241</v>
@@ -5330,10 +5330,10 @@
         <v>49</v>
       </c>
       <c r="C158" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D158" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="E158" s="4" t="s">
         <v>241</v>
@@ -5347,10 +5347,10 @@
         <v>49</v>
       </c>
       <c r="C159" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D159" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="E159" s="4" t="s">
         <v>242</v>
@@ -5364,10 +5364,10 @@
         <v>49</v>
       </c>
       <c r="C160" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D160" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="E160" s="4" t="s">
         <v>242</v>
@@ -5381,10 +5381,10 @@
         <v>49</v>
       </c>
       <c r="C161" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="D161" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="E161" s="4" t="s">
         <v>242</v>
@@ -5398,10 +5398,10 @@
         <v>49</v>
       </c>
       <c r="C162" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D162" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="E162" s="4" t="s">
         <v>241</v>
@@ -5415,10 +5415,10 @@
         <v>49</v>
       </c>
       <c r="C163" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D163" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="E163" s="4" t="s">
         <v>241</v>
@@ -5432,10 +5432,10 @@
         <v>49</v>
       </c>
       <c r="C164" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D164" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="E164" s="4" t="s">
         <v>241</v>
@@ -5449,10 +5449,10 @@
         <v>49</v>
       </c>
       <c r="C165" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D165" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="E165" s="4" t="s">
         <v>241</v>
@@ -5472,10 +5472,10 @@
         <v>49</v>
       </c>
       <c r="C166" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D166" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="E166" s="4" t="s">
         <v>241</v>
@@ -5495,10 +5495,10 @@
         <v>49</v>
       </c>
       <c r="C167" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D167" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="E167" s="4" t="s">
         <v>241</v>
@@ -6232,10 +6232,10 @@
         <v>65</v>
       </c>
       <c r="C210" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D210" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="E210" s="4" t="s">
         <v>274</v>
@@ -6249,10 +6249,10 @@
         <v>65</v>
       </c>
       <c r="C211" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="D211" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="E211" s="4" t="s">
         <v>274</v>
@@ -6266,10 +6266,10 @@
         <v>65</v>
       </c>
       <c r="C212" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D212" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="E212" s="4" t="s">
         <v>274</v>
@@ -6283,10 +6283,10 @@
         <v>65</v>
       </c>
       <c r="C213" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D213" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E213" s="4" t="s">
         <v>274</v>
@@ -6300,10 +6300,10 @@
         <v>65</v>
       </c>
       <c r="C214" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D214" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="E214" s="4" t="s">
         <v>274</v>
@@ -6317,10 +6317,10 @@
         <v>65</v>
       </c>
       <c r="C215" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D215" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="E215" s="4" t="s">
         <v>274</v>
@@ -6334,10 +6334,10 @@
         <v>65</v>
       </c>
       <c r="C216" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D216" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="E216" s="4" t="s">
         <v>274</v>
@@ -6354,10 +6354,10 @@
         <v>65</v>
       </c>
       <c r="C217" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D217" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="E217" s="4" t="s">
         <v>274</v>
@@ -6374,10 +6374,10 @@
         <v>65</v>
       </c>
       <c r="C218" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D218" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="E218" s="4" t="s">
         <v>274</v>
@@ -6654,7 +6654,7 @@
         <v>302</v>
       </c>
       <c r="E232" s="4" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="233" spans="1:12" x14ac:dyDescent="0.25">
@@ -6665,13 +6665,13 @@
         <v>317</v>
       </c>
       <c r="C233" t="s">
+        <v>330</v>
+      </c>
+      <c r="D233" t="s">
+        <v>331</v>
+      </c>
+      <c r="E233" s="4" t="s">
         <v>334</v>
-      </c>
-      <c r="D233" t="s">
-        <v>335</v>
-      </c>
-      <c r="E233" s="4" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="234" spans="1:12" x14ac:dyDescent="0.25">
@@ -6685,13 +6685,13 @@
         <v>11</v>
       </c>
       <c r="D234" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E234" s="4" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="F234" s="4" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
     </row>
     <row r="235" spans="1:12" x14ac:dyDescent="0.25">
@@ -6699,16 +6699,16 @@
         <v>299</v>
       </c>
       <c r="B235" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C235" t="s">
         <v>6</v>
       </c>
       <c r="D235" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="E235" s="4" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
     </row>
     <row r="236" spans="1:12" x14ac:dyDescent="0.25">
@@ -6716,19 +6716,19 @@
         <v>299</v>
       </c>
       <c r="B236" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C236" t="s">
         <v>11</v>
       </c>
       <c r="D236" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E236" s="6" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="F236" s="6" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="237" spans="1:12" x14ac:dyDescent="0.25">
@@ -6745,10 +6745,10 @@
         <v>303</v>
       </c>
       <c r="E237" s="6" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="F237" s="6" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
     </row>
     <row r="238" spans="1:12" x14ac:dyDescent="0.25">
@@ -6762,420 +6762,403 @@
         <v>10</v>
       </c>
       <c r="D238" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="E238" s="6" t="s">
-        <v>349</v>
+        <v>345</v>
+      </c>
+    </row>
+    <row r="239" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>299</v>
+      </c>
+      <c r="B239" t="s">
+        <v>93</v>
+      </c>
+      <c r="C239" t="s">
+        <v>6</v>
+      </c>
+      <c r="D239" t="s">
+        <v>631</v>
+      </c>
+      <c r="E239" s="4" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="240" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A240" s="7" t="s">
+      <c r="A240" t="s">
+        <v>299</v>
+      </c>
+      <c r="B240" t="s">
+        <v>93</v>
+      </c>
+      <c r="C240" t="s">
+        <v>7</v>
+      </c>
+      <c r="D240" t="s">
+        <v>632</v>
+      </c>
+      <c r="E240" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F240" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>299</v>
+      </c>
+      <c r="B241" t="s">
+        <v>93</v>
+      </c>
+      <c r="C241" t="s">
+        <v>10</v>
+      </c>
+      <c r="D241" t="s">
+        <v>633</v>
+      </c>
+      <c r="E241" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>299</v>
+      </c>
+      <c r="B242" t="s">
+        <v>93</v>
+      </c>
+      <c r="C242" t="s">
+        <v>11</v>
+      </c>
+      <c r="D242" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="E242" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F242" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="243" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E243" s="6"/>
+    </row>
+    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A245" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="B240" s="7"/>
-      <c r="C240" s="7"/>
-      <c r="D240" s="7"/>
-      <c r="E240" s="7"/>
-      <c r="F240" s="7"/>
-      <c r="G240" s="7"/>
-      <c r="H240" s="7"/>
-      <c r="I240" s="7"/>
-      <c r="J240" s="7"/>
-      <c r="K240" s="7"/>
-      <c r="L240" s="7"/>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A241" t="s">
-        <v>300</v>
-      </c>
-      <c r="B241" t="s">
-        <v>300</v>
-      </c>
-      <c r="C241" t="s">
-        <v>6</v>
-      </c>
-      <c r="D241" t="s">
-        <v>304</v>
-      </c>
-      <c r="E241" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A242" t="s">
-        <v>300</v>
-      </c>
-      <c r="B242" t="s">
-        <v>300</v>
-      </c>
-      <c r="C242" t="s">
-        <v>334</v>
-      </c>
-      <c r="D242" t="s">
-        <v>350</v>
-      </c>
-      <c r="E242" s="6" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A243" t="s">
-        <v>300</v>
-      </c>
-      <c r="B243" t="s">
-        <v>300</v>
-      </c>
-      <c r="C243" t="s">
-        <v>11</v>
-      </c>
-      <c r="D243" t="s">
-        <v>351</v>
-      </c>
-      <c r="E243" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="F243" s="6" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A244" t="s">
-        <v>300</v>
-      </c>
-      <c r="B244" t="s">
-        <v>308</v>
-      </c>
-      <c r="C244" t="s">
-        <v>6</v>
-      </c>
-      <c r="D244" t="s">
-        <v>305</v>
-      </c>
-      <c r="E244" s="6" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A245" t="s">
-        <v>300</v>
-      </c>
-      <c r="B245" t="s">
-        <v>308</v>
-      </c>
-      <c r="C245" t="s">
-        <v>334</v>
-      </c>
-      <c r="D245" t="s">
-        <v>355</v>
-      </c>
-      <c r="E245" s="6" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B245" s="7"/>
+      <c r="C245" s="7"/>
+      <c r="D245" s="7"/>
+      <c r="E245" s="7"/>
+      <c r="F245" s="7"/>
+      <c r="G245" s="7"/>
+      <c r="H245" s="7"/>
+      <c r="I245" s="7"/>
+      <c r="J245" s="7"/>
+      <c r="K245" s="7"/>
+      <c r="L245" s="7"/>
+    </row>
+    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>300</v>
       </c>
       <c r="B246" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C246" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D246" t="s">
-        <v>356</v>
+        <v>304</v>
       </c>
       <c r="E246" s="6" t="s">
-        <v>359</v>
-      </c>
-      <c r="F246" s="6" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="247" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>300</v>
       </c>
       <c r="B247" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C247" t="s">
-        <v>10</v>
+        <v>330</v>
       </c>
       <c r="D247" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="E247" s="6" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>300</v>
       </c>
       <c r="B248" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="C248" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D248" t="s">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="E248" s="6" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+      <c r="F248" s="6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>300</v>
       </c>
       <c r="B249" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C249" t="s">
-        <v>334</v>
+        <v>6</v>
       </c>
       <c r="D249" t="s">
-        <v>361</v>
+        <v>305</v>
       </c>
       <c r="E249" s="6" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>300</v>
       </c>
       <c r="B250" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C250" t="s">
-        <v>11</v>
+        <v>330</v>
       </c>
       <c r="D250" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="E250" s="6" t="s">
-        <v>365</v>
-      </c>
-      <c r="F250" s="6" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="251" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>300</v>
       </c>
       <c r="B251" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C251" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D251" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="E251" s="6" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+      <c r="F251" s="6" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>300</v>
       </c>
       <c r="B252" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C252" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D252" t="s">
-        <v>306</v>
+        <v>353</v>
       </c>
       <c r="E252" s="6" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>300</v>
       </c>
       <c r="B253" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C253" t="s">
-        <v>334</v>
+        <v>6</v>
       </c>
       <c r="D253" t="s">
-        <v>367</v>
+        <v>307</v>
       </c>
       <c r="E253" s="6" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="254" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>300</v>
       </c>
       <c r="B254" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C254" t="s">
-        <v>11</v>
+        <v>330</v>
       </c>
       <c r="D254" t="s">
-        <v>420</v>
+        <v>357</v>
       </c>
       <c r="E254" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="F254" s="6" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>300</v>
       </c>
       <c r="B255" t="s">
+        <v>310</v>
+      </c>
+      <c r="C255" t="s">
+        <v>11</v>
+      </c>
+      <c r="D255" t="s">
+        <v>358</v>
+      </c>
+      <c r="E255" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="F255" s="6" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="256" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>300</v>
+      </c>
+      <c r="B256" t="s">
+        <v>310</v>
+      </c>
+      <c r="C256" t="s">
+        <v>10</v>
+      </c>
+      <c r="D256" t="s">
+        <v>359</v>
+      </c>
+      <c r="E256" s="6" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>300</v>
+      </c>
+      <c r="B257" t="s">
         <v>309</v>
       </c>
-      <c r="C255" t="s">
-        <v>10</v>
-      </c>
-      <c r="D255" t="s">
-        <v>368</v>
-      </c>
-      <c r="E255" s="6" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A257" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="B257" s="9"/>
-      <c r="C257" s="9"/>
-      <c r="D257" s="9"/>
-      <c r="E257" s="9"/>
-      <c r="F257" s="9"/>
-      <c r="G257" s="9"/>
-      <c r="H257" s="9"/>
-      <c r="I257" s="9"/>
-      <c r="J257" s="9"/>
-      <c r="K257" s="9"/>
-      <c r="L257" s="10"/>
+      <c r="C257" t="s">
+        <v>6</v>
+      </c>
+      <c r="D257" t="s">
+        <v>306</v>
+      </c>
+      <c r="E257" s="6" t="s">
+        <v>365</v>
+      </c>
     </row>
     <row r="258" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B258" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C258" t="s">
-        <v>6</v>
+        <v>330</v>
       </c>
       <c r="D258" t="s">
-        <v>311</v>
+        <v>363</v>
       </c>
       <c r="E258" s="6" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
     </row>
     <row r="259" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B259" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C259" t="s">
-        <v>334</v>
+        <v>11</v>
       </c>
       <c r="D259" t="s">
-        <v>372</v>
+        <v>416</v>
       </c>
       <c r="E259" s="6" t="s">
-        <v>375</v>
+        <v>366</v>
+      </c>
+      <c r="F259" s="6" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="260" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
+        <v>300</v>
+      </c>
+      <c r="B260" t="s">
+        <v>309</v>
+      </c>
+      <c r="C260" t="s">
+        <v>10</v>
+      </c>
+      <c r="D260" t="s">
+        <v>364</v>
+      </c>
+      <c r="E260" s="6" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A262" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="B260" t="s">
-        <v>312</v>
-      </c>
-      <c r="C260" t="s">
-        <v>11</v>
-      </c>
-      <c r="D260" t="s">
-        <v>373</v>
-      </c>
-      <c r="E260" s="6" t="s">
-        <v>375</v>
-      </c>
-      <c r="F260" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="G260" s="6" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A261" t="s">
-        <v>301</v>
-      </c>
-      <c r="B261" t="s">
-        <v>313</v>
-      </c>
-      <c r="C261" t="s">
-        <v>6</v>
-      </c>
-      <c r="D261" t="s">
-        <v>378</v>
-      </c>
-      <c r="E261" s="6" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A262" t="s">
-        <v>301</v>
-      </c>
-      <c r="B262" t="s">
-        <v>313</v>
-      </c>
-      <c r="C262" t="s">
-        <v>334</v>
-      </c>
-      <c r="D262" t="s">
-        <v>379</v>
-      </c>
-      <c r="E262" s="6" t="s">
-        <v>383</v>
-      </c>
+      <c r="B262" s="11"/>
+      <c r="C262" s="11"/>
+      <c r="D262" s="11"/>
+      <c r="E262" s="11"/>
+      <c r="F262" s="11"/>
+      <c r="G262" s="11"/>
+      <c r="H262" s="11"/>
+      <c r="I262" s="11"/>
+      <c r="J262" s="11"/>
+      <c r="K262" s="11"/>
+      <c r="L262" s="12"/>
     </row>
     <row r="263" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>301</v>
       </c>
       <c r="B263" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C263" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D263" t="s">
-        <v>380</v>
+        <v>311</v>
       </c>
       <c r="E263" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="F263" s="6" t="s">
-        <v>385</v>
+        <v>370</v>
       </c>
     </row>
     <row r="264" spans="1:12" x14ac:dyDescent="0.25">
@@ -7183,16 +7166,16 @@
         <v>301</v>
       </c>
       <c r="B264" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C264" t="s">
-        <v>10</v>
+        <v>330</v>
       </c>
       <c r="D264" t="s">
-        <v>381</v>
+        <v>368</v>
       </c>
       <c r="E264" s="6" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
     </row>
     <row r="265" spans="1:12" x14ac:dyDescent="0.25">
@@ -7200,16 +7183,22 @@
         <v>301</v>
       </c>
       <c r="B265" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C265" t="s">
         <v>11</v>
       </c>
       <c r="D265" t="s">
-        <v>386</v>
+        <v>369</v>
       </c>
       <c r="E265" s="6" t="s">
-        <v>387</v>
+        <v>371</v>
+      </c>
+      <c r="F265" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="G265" s="6" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="266" spans="1:12" x14ac:dyDescent="0.25">
@@ -7217,16 +7206,16 @@
         <v>301</v>
       </c>
       <c r="B266" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C266" t="s">
         <v>6</v>
       </c>
       <c r="D266" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="E266" s="6" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
     </row>
     <row r="267" spans="1:12" x14ac:dyDescent="0.25">
@@ -7234,16 +7223,16 @@
         <v>301</v>
       </c>
       <c r="B267" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C267" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D267" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="E267" s="6" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
     </row>
     <row r="268" spans="1:12" x14ac:dyDescent="0.25">
@@ -7251,19 +7240,19 @@
         <v>301</v>
       </c>
       <c r="B268" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C268" t="s">
         <v>11</v>
       </c>
       <c r="D268" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="E268" s="6" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="F268" s="6" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
     </row>
     <row r="269" spans="1:12" x14ac:dyDescent="0.25">
@@ -7271,262 +7260,191 @@
         <v>301</v>
       </c>
       <c r="B269" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C269" t="s">
         <v>10</v>
       </c>
       <c r="D269" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="E269" s="6" t="s">
-        <v>393</v>
+        <v>379</v>
+      </c>
+    </row>
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>301</v>
+      </c>
+      <c r="B270" t="s">
+        <v>314</v>
+      </c>
+      <c r="C270" t="s">
+        <v>11</v>
+      </c>
+      <c r="D270" t="s">
+        <v>382</v>
+      </c>
+      <c r="E270" s="6" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="271" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A271" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="B271" s="7"/>
-      <c r="C271" s="7"/>
-      <c r="D271" s="7"/>
-      <c r="E271" s="7"/>
-      <c r="F271" s="7"/>
-      <c r="G271" s="7"/>
-      <c r="H271" s="7"/>
-      <c r="I271" s="7"/>
-      <c r="J271" s="7"/>
-      <c r="K271" s="7"/>
-      <c r="L271" s="7"/>
+      <c r="A271" t="s">
+        <v>301</v>
+      </c>
+      <c r="B271" t="s">
+        <v>315</v>
+      </c>
+      <c r="C271" t="s">
+        <v>6</v>
+      </c>
+      <c r="D271" t="s">
+        <v>384</v>
+      </c>
+      <c r="E271" s="6" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="272" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="B272" t="s">
-        <v>93</v>
+        <v>315</v>
       </c>
       <c r="C272" t="s">
-        <v>6</v>
+        <v>330</v>
       </c>
       <c r="D272" t="s">
-        <v>320</v>
-      </c>
-      <c r="E272" s="4" t="s">
-        <v>197</v>
+        <v>385</v>
+      </c>
+      <c r="E272" s="6" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="273" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="B273" t="s">
-        <v>93</v>
+        <v>315</v>
       </c>
       <c r="C273" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D273" t="s">
-        <v>321</v>
-      </c>
-      <c r="E273" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F273" s="4" t="s">
-        <v>200</v>
+        <v>387</v>
+      </c>
+      <c r="E273" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="F273" s="6" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="274" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="B274" t="s">
-        <v>93</v>
+        <v>315</v>
       </c>
       <c r="C274" t="s">
         <v>10</v>
       </c>
       <c r="D274" t="s">
-        <v>322</v>
-      </c>
-      <c r="E274" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A275" t="s">
-        <v>319</v>
-      </c>
-      <c r="B275" t="s">
-        <v>93</v>
-      </c>
-      <c r="C275" t="s">
-        <v>11</v>
-      </c>
-      <c r="D275" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="E275" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>199</v>
+        <v>386</v>
+      </c>
+      <c r="E274" s="6" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="276" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A276" t="s">
-        <v>319</v>
-      </c>
-      <c r="B276" t="s">
-        <v>94</v>
-      </c>
-      <c r="C276" t="s">
-        <v>6</v>
-      </c>
-      <c r="D276" t="s">
-        <v>324</v>
-      </c>
-      <c r="E276" s="4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="277" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A277" t="s">
-        <v>319</v>
-      </c>
-      <c r="B277" t="s">
-        <v>94</v>
-      </c>
-      <c r="C277" t="s">
-        <v>7</v>
-      </c>
-      <c r="D277" t="s">
-        <v>325</v>
-      </c>
-      <c r="E277" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A278" t="s">
-        <v>319</v>
-      </c>
-      <c r="B278" t="s">
-        <v>94</v>
-      </c>
-      <c r="C278" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D278" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="E278" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="F278" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A280" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B280" s="7"/>
-      <c r="C280" s="7"/>
-      <c r="D280" s="7"/>
-      <c r="E280" s="7"/>
-      <c r="F280" s="7"/>
-      <c r="G280" s="7"/>
-      <c r="H280" s="7"/>
-      <c r="I280" s="7"/>
-      <c r="J280" s="7"/>
-      <c r="K280" s="7"/>
-      <c r="L280" s="7"/>
+      <c r="A276" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="B276" s="7"/>
+      <c r="C276" s="7"/>
+      <c r="D276" s="7"/>
+      <c r="E276" s="7"/>
+      <c r="F276" s="7"/>
+      <c r="G276" s="7"/>
+      <c r="H276" s="7"/>
+      <c r="I276" s="7"/>
+      <c r="J276" s="7"/>
+      <c r="K276" s="7"/>
+      <c r="L276" s="7"/>
     </row>
     <row r="281" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>39</v>
+        <v>319</v>
       </c>
       <c r="B281" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="C281" t="s">
         <v>6</v>
       </c>
       <c r="D281" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="E281" s="4" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
     </row>
     <row r="282" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>39</v>
+        <v>319</v>
       </c>
       <c r="B282" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="C282" t="s">
-        <v>430</v>
+        <v>7</v>
       </c>
       <c r="D282" t="s">
-        <v>562</v>
+        <v>321</v>
       </c>
       <c r="E282" s="4" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
     </row>
     <row r="283" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
+        <v>319</v>
+      </c>
+      <c r="B283" t="s">
+        <v>94</v>
+      </c>
+      <c r="C283" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D283" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E283" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F283" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A285" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B283" t="s">
-        <v>39</v>
-      </c>
-      <c r="C283" t="s">
-        <v>431</v>
-      </c>
-      <c r="D283" t="s">
-        <v>563</v>
-      </c>
-      <c r="E283" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A284" t="s">
-        <v>39</v>
-      </c>
-      <c r="B284" t="s">
-        <v>39</v>
-      </c>
-      <c r="C284" t="s">
-        <v>432</v>
-      </c>
-      <c r="D284" t="s">
-        <v>564</v>
-      </c>
-      <c r="E284" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A285" t="s">
-        <v>39</v>
-      </c>
-      <c r="B285" t="s">
-        <v>39</v>
-      </c>
-      <c r="C285" t="s">
-        <v>442</v>
-      </c>
-      <c r="D285" t="s">
-        <v>565</v>
-      </c>
-      <c r="E285" s="4" t="s">
-        <v>219</v>
-      </c>
+      <c r="B285" s="7"/>
+      <c r="C285" s="7"/>
+      <c r="D285" s="7"/>
+      <c r="E285" s="7"/>
+      <c r="F285" s="7"/>
+      <c r="G285" s="7"/>
+      <c r="H285" s="7"/>
+      <c r="I285" s="7"/>
+      <c r="J285" s="7"/>
+      <c r="K285" s="7"/>
+      <c r="L285" s="7"/>
     </row>
     <row r="286" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
@@ -7536,13 +7454,13 @@
         <v>39</v>
       </c>
       <c r="C286" t="s">
-        <v>443</v>
+        <v>6</v>
       </c>
       <c r="D286" t="s">
-        <v>566</v>
+        <v>323</v>
       </c>
       <c r="E286" s="4" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="287" spans="1:12" x14ac:dyDescent="0.25">
@@ -7553,13 +7471,13 @@
         <v>39</v>
       </c>
       <c r="C287" t="s">
-        <v>444</v>
+        <v>426</v>
       </c>
       <c r="D287" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
       <c r="E287" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="288" spans="1:12" x14ac:dyDescent="0.25">
@@ -7570,10 +7488,10 @@
         <v>39</v>
       </c>
       <c r="C288" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="D288" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
       <c r="E288" s="4" t="s">
         <v>218</v>
@@ -7587,10 +7505,10 @@
         <v>39</v>
       </c>
       <c r="C289" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="D289" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
       <c r="E289" s="4" t="s">
         <v>218</v>
@@ -7607,10 +7525,10 @@
         <v>438</v>
       </c>
       <c r="D290" t="s">
-        <v>570</v>
+        <v>561</v>
       </c>
       <c r="E290" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="291" spans="1:8" x14ac:dyDescent="0.25">
@@ -7621,22 +7539,13 @@
         <v>39</v>
       </c>
       <c r="C291" t="s">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="D291" t="s">
-        <v>571</v>
+        <v>562</v>
       </c>
       <c r="E291" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="F291" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="G291" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H291" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="292" spans="1:8" x14ac:dyDescent="0.25">
@@ -7647,22 +7556,13 @@
         <v>39</v>
       </c>
       <c r="C292" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="D292" t="s">
-        <v>572</v>
+        <v>563</v>
       </c>
       <c r="E292" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="F292" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="G292" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H292" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="293" spans="1:8" x14ac:dyDescent="0.25">
@@ -7673,22 +7573,13 @@
         <v>39</v>
       </c>
       <c r="C293" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="D293" t="s">
-        <v>573</v>
+        <v>564</v>
       </c>
       <c r="E293" s="4" t="s">
         <v>218</v>
-      </c>
-      <c r="F293" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="G293" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H293" s="4" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="294" spans="1:8" x14ac:dyDescent="0.25">
@@ -7699,16 +7590,13 @@
         <v>39</v>
       </c>
       <c r="C294" t="s">
-        <v>22</v>
+        <v>433</v>
       </c>
       <c r="D294" t="s">
-        <v>328</v>
+        <v>565</v>
       </c>
       <c r="E294" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="F294" s="4" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="295" spans="1:8" x14ac:dyDescent="0.25">
@@ -7716,16 +7604,16 @@
         <v>39</v>
       </c>
       <c r="B295" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C295" t="s">
-        <v>6</v>
+        <v>434</v>
       </c>
       <c r="D295" t="s">
-        <v>329</v>
+        <v>566</v>
       </c>
       <c r="E295" s="4" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="296" spans="1:8" x14ac:dyDescent="0.25">
@@ -7733,16 +7621,25 @@
         <v>39</v>
       </c>
       <c r="B296" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C296" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="D296" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="E296" s="4" t="s">
-        <v>225</v>
+        <v>218</v>
+      </c>
+      <c r="F296" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G296" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H296" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="297" spans="1:8" x14ac:dyDescent="0.25">
@@ -7750,16 +7647,25 @@
         <v>39</v>
       </c>
       <c r="B297" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C297" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
       <c r="D297" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="E297" s="4" t="s">
-        <v>225</v>
+        <v>218</v>
+      </c>
+      <c r="F297" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G297" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H297" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="298" spans="1:8" x14ac:dyDescent="0.25">
@@ -7767,16 +7673,25 @@
         <v>39</v>
       </c>
       <c r="B298" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C298" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
       <c r="D298" t="s">
-        <v>576</v>
+        <v>569</v>
       </c>
       <c r="E298" s="4" t="s">
-        <v>225</v>
+        <v>218</v>
+      </c>
+      <c r="F298" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G298" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H298" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="299" spans="1:8" x14ac:dyDescent="0.25">
@@ -7784,16 +7699,19 @@
         <v>39</v>
       </c>
       <c r="B299" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C299" t="s">
-        <v>436</v>
+        <v>22</v>
       </c>
       <c r="D299" t="s">
-        <v>577</v>
+        <v>324</v>
       </c>
       <c r="E299" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
+      </c>
+      <c r="F299" s="4" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="300" spans="1:8" x14ac:dyDescent="0.25">
@@ -7804,13 +7722,13 @@
         <v>40</v>
       </c>
       <c r="C300" t="s">
-        <v>437</v>
+        <v>6</v>
       </c>
       <c r="D300" t="s">
-        <v>578</v>
+        <v>325</v>
       </c>
       <c r="E300" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="301" spans="1:8" x14ac:dyDescent="0.25">
@@ -7821,13 +7739,13 @@
         <v>40</v>
       </c>
       <c r="C301" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
       <c r="D301" t="s">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="E301" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.25">
@@ -7838,19 +7756,13 @@
         <v>40</v>
       </c>
       <c r="C302" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D302" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="E302" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="F302" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="G302" s="4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.25">
@@ -7861,19 +7773,13 @@
         <v>40</v>
       </c>
       <c r="C303" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D303" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="E303" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="F303" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="G303" s="4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.25">
@@ -7884,19 +7790,13 @@
         <v>40</v>
       </c>
       <c r="C304" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="D304" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="E304" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="F304" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="G304" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="305" spans="1:12" x14ac:dyDescent="0.25">
@@ -7907,16 +7807,13 @@
         <v>40</v>
       </c>
       <c r="C305" t="s">
-        <v>22</v>
+        <v>433</v>
       </c>
       <c r="D305" t="s">
-        <v>330</v>
+        <v>574</v>
       </c>
       <c r="E305" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="F305" s="4" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="306" spans="1:12" x14ac:dyDescent="0.25">
@@ -7927,874 +7824,980 @@
         <v>40</v>
       </c>
       <c r="C306" t="s">
-        <v>26</v>
+        <v>434</v>
       </c>
       <c r="D306" t="s">
-        <v>331</v>
+        <v>575</v>
       </c>
       <c r="E306" s="4" t="s">
-        <v>232</v>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="307" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>39</v>
+      </c>
+      <c r="B307" t="s">
+        <v>40</v>
+      </c>
+      <c r="C307" t="s">
+        <v>420</v>
+      </c>
+      <c r="D307" t="s">
+        <v>576</v>
+      </c>
+      <c r="E307" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F307" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="G307" s="4" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="308" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A308" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="B308" s="7"/>
-      <c r="C308" s="7"/>
-      <c r="D308" s="7"/>
-      <c r="E308" s="7"/>
-      <c r="F308" s="7"/>
-      <c r="G308" s="7"/>
-      <c r="H308" s="7"/>
-      <c r="I308" s="7"/>
-      <c r="J308" s="7"/>
-      <c r="K308" s="7"/>
-      <c r="L308" s="7"/>
+      <c r="A308" t="s">
+        <v>39</v>
+      </c>
+      <c r="B308" t="s">
+        <v>40</v>
+      </c>
+      <c r="C308" t="s">
+        <v>421</v>
+      </c>
+      <c r="D308" t="s">
+        <v>577</v>
+      </c>
+      <c r="E308" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F308" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="G308" s="4" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="309" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>332</v>
+        <v>39</v>
       </c>
       <c r="B309" t="s">
-        <v>395</v>
+        <v>40</v>
       </c>
       <c r="C309" t="s">
-        <v>11</v>
+        <v>422</v>
       </c>
       <c r="D309" t="s">
-        <v>396</v>
-      </c>
-      <c r="E309" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="F309" s="5" t="s">
-        <v>401</v>
+        <v>578</v>
+      </c>
+      <c r="E309" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F309" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="G309" s="4" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="310" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>332</v>
+        <v>39</v>
       </c>
       <c r="B310" t="s">
-        <v>398</v>
+        <v>40</v>
       </c>
       <c r="C310" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D310" t="s">
-        <v>399</v>
-      </c>
-      <c r="E310" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="F310" s="5" t="s">
-        <v>402</v>
+        <v>326</v>
+      </c>
+      <c r="E310" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F310" s="4" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="311" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>332</v>
+        <v>39</v>
       </c>
       <c r="B311" t="s">
-        <v>403</v>
+        <v>40</v>
       </c>
       <c r="C311" t="s">
+        <v>26</v>
+      </c>
+      <c r="D311" t="s">
+        <v>327</v>
+      </c>
+      <c r="E311" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A313" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="B313" s="7"/>
+      <c r="C313" s="7"/>
+      <c r="D313" s="7"/>
+      <c r="E313" s="7"/>
+      <c r="F313" s="7"/>
+      <c r="G313" s="7"/>
+      <c r="H313" s="7"/>
+      <c r="I313" s="7"/>
+      <c r="J313" s="7"/>
+      <c r="K313" s="7"/>
+      <c r="L313" s="7"/>
+    </row>
+    <row r="314" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>328</v>
+      </c>
+      <c r="B314" t="s">
+        <v>391</v>
+      </c>
+      <c r="C314" t="s">
         <v>11</v>
       </c>
-      <c r="D311" t="s">
-        <v>404</v>
-      </c>
-      <c r="E311" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="F311" s="5" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="312" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A312" t="s">
-        <v>332</v>
-      </c>
-      <c r="B312" t="s">
-        <v>407</v>
-      </c>
-      <c r="C312" t="s">
+      <c r="D314" t="s">
+        <v>392</v>
+      </c>
+      <c r="E314" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="F314" s="5" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A315" t="s">
+        <v>328</v>
+      </c>
+      <c r="B315" t="s">
+        <v>394</v>
+      </c>
+      <c r="C315" t="s">
         <v>11</v>
       </c>
-      <c r="D312" t="s">
-        <v>408</v>
-      </c>
-      <c r="E312" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="F312" s="5" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A313" t="s">
-        <v>332</v>
-      </c>
-      <c r="B313" t="s">
-        <v>411</v>
-      </c>
-      <c r="C313" t="s">
-        <v>11</v>
-      </c>
-      <c r="D313" t="s">
-        <v>412</v>
-      </c>
-      <c r="E313" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="F313" s="5" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A315" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="B315" s="7"/>
-      <c r="C315" s="7"/>
-      <c r="D315" s="7"/>
-      <c r="E315" s="7"/>
-      <c r="F315" s="7"/>
-      <c r="G315" s="7"/>
-      <c r="H315" s="7"/>
-      <c r="I315" s="7"/>
-      <c r="J315" s="7"/>
-      <c r="K315" s="7"/>
-      <c r="L315" s="7"/>
+      <c r="D315" t="s">
+        <v>395</v>
+      </c>
+      <c r="E315" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="F315" s="5" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="316" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>586</v>
+        <v>328</v>
       </c>
       <c r="B316" t="s">
-        <v>5</v>
+        <v>399</v>
       </c>
       <c r="C316" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D316" t="s">
-        <v>589</v>
+        <v>400</v>
       </c>
       <c r="E316" s="5" t="s">
-        <v>415</v>
+        <v>401</v>
+      </c>
+      <c r="F316" s="5" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="317" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>586</v>
+        <v>328</v>
       </c>
       <c r="B317" t="s">
-        <v>5</v>
+        <v>403</v>
       </c>
       <c r="C317" t="s">
-        <v>583</v>
+        <v>11</v>
       </c>
       <c r="D317" t="s">
-        <v>590</v>
+        <v>404</v>
       </c>
       <c r="E317" s="5" t="s">
-        <v>416</v>
+        <v>405</v>
+      </c>
+      <c r="F317" s="5" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="318" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>586</v>
+        <v>328</v>
       </c>
       <c r="B318" t="s">
-        <v>5</v>
+        <v>407</v>
       </c>
       <c r="C318" t="s">
-        <v>584</v>
+        <v>11</v>
       </c>
       <c r="D318" t="s">
-        <v>591</v>
+        <v>408</v>
       </c>
       <c r="E318" s="5" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="319" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A319" t="s">
-        <v>586</v>
-      </c>
-      <c r="B319" t="s">
-        <v>5</v>
-      </c>
-      <c r="C319" t="s">
-        <v>585</v>
-      </c>
-      <c r="D319" t="s">
-        <v>592</v>
-      </c>
-      <c r="E319" s="5" t="s">
-        <v>416</v>
+        <v>409</v>
+      </c>
+      <c r="F318" s="5" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="320" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A320" t="s">
-        <v>586</v>
-      </c>
-      <c r="B320" t="s">
-        <v>5</v>
-      </c>
-      <c r="C320" t="s">
-        <v>424</v>
-      </c>
-      <c r="D320" t="s">
-        <v>593</v>
-      </c>
-      <c r="E320" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F320" s="5" t="s">
-        <v>419</v>
-      </c>
+      <c r="A320" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="B320" s="7"/>
+      <c r="C320" s="7"/>
+      <c r="D320" s="7"/>
+      <c r="E320" s="7"/>
+      <c r="F320" s="7"/>
+      <c r="G320" s="7"/>
+      <c r="H320" s="7"/>
+      <c r="I320" s="7"/>
+      <c r="J320" s="7"/>
+      <c r="K320" s="7"/>
+      <c r="L320" s="7"/>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B321" t="s">
         <v>5</v>
       </c>
       <c r="C321" t="s">
-        <v>425</v>
+        <v>6</v>
       </c>
       <c r="D321" t="s">
-        <v>594</v>
+        <v>585</v>
       </c>
       <c r="E321" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F321" s="5" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B322" t="s">
         <v>5</v>
       </c>
       <c r="C322" t="s">
-        <v>426</v>
+        <v>579</v>
       </c>
       <c r="D322" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
       <c r="E322" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F322" s="5" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B323" t="s">
         <v>5</v>
       </c>
       <c r="C323" t="s">
-        <v>436</v>
+        <v>580</v>
       </c>
       <c r="D323" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
       <c r="E323" s="5" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B324" t="s">
         <v>5</v>
       </c>
       <c r="C324" t="s">
-        <v>437</v>
+        <v>581</v>
       </c>
       <c r="D324" t="s">
-        <v>597</v>
+        <v>588</v>
       </c>
       <c r="E324" s="5" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B325" t="s">
         <v>5</v>
       </c>
       <c r="C325" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="D325" t="s">
-        <v>598</v>
+        <v>589</v>
       </c>
       <c r="E325" s="5" t="s">
-        <v>418</v>
+        <v>413</v>
+      </c>
+      <c r="F325" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B326" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C326" t="s">
-        <v>6</v>
+        <v>421</v>
       </c>
       <c r="D326" t="s">
-        <v>599</v>
+        <v>590</v>
       </c>
       <c r="E326" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="F326" s="5" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="327" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B327" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C327" t="s">
-        <v>583</v>
+        <v>422</v>
       </c>
       <c r="D327" t="s">
-        <v>600</v>
+        <v>591</v>
       </c>
       <c r="E327" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
+      </c>
+      <c r="F327" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B328" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C328" t="s">
-        <v>584</v>
+        <v>432</v>
       </c>
       <c r="D328" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
       <c r="E328" s="5" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B329" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C329" t="s">
-        <v>585</v>
+        <v>433</v>
       </c>
       <c r="D329" t="s">
-        <v>602</v>
+        <v>593</v>
       </c>
       <c r="E329" s="5" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B330" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C330" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="D330" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E330" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F330" s="5" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B331" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C331" t="s">
-        <v>425</v>
+        <v>6</v>
       </c>
       <c r="D331" t="s">
-        <v>604</v>
+        <v>595</v>
       </c>
       <c r="E331" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F331" s="5" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B332" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C332" t="s">
-        <v>426</v>
+        <v>579</v>
       </c>
       <c r="D332" t="s">
-        <v>605</v>
+        <v>596</v>
       </c>
       <c r="E332" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="F332" s="5" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B333" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C333" t="s">
-        <v>436</v>
+        <v>580</v>
       </c>
       <c r="D333" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="E333" s="5" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B334" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C334" t="s">
-        <v>437</v>
+        <v>581</v>
       </c>
       <c r="D334" t="s">
-        <v>607</v>
+        <v>598</v>
       </c>
       <c r="E334" s="5" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B335" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C335" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="D335" t="s">
-        <v>608</v>
+        <v>599</v>
       </c>
       <c r="E335" s="5" t="s">
-        <v>418</v>
+        <v>413</v>
+      </c>
+      <c r="F335" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B336" t="s">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C336" t="s">
-        <v>6</v>
+        <v>421</v>
       </c>
       <c r="D336" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="E336" s="5" t="s">
-        <v>629</v>
+        <v>413</v>
+      </c>
+      <c r="F336" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B337" t="s">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C337" t="s">
-        <v>583</v>
+        <v>422</v>
       </c>
       <c r="D337" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="E337" s="5" t="s">
-        <v>631</v>
+        <v>413</v>
+      </c>
+      <c r="F337" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B338" t="s">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C338" t="s">
-        <v>584</v>
+        <v>432</v>
       </c>
       <c r="D338" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="E338" s="5" t="s">
-        <v>631</v>
+        <v>414</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B339" t="s">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C339" t="s">
-        <v>585</v>
+        <v>433</v>
       </c>
       <c r="D339" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="E339" s="5" t="s">
-        <v>631</v>
+        <v>414</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B340" t="s">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C340" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="D340" t="s">
-        <v>613</v>
+        <v>604</v>
       </c>
       <c r="E340" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="F340" s="5" t="s">
-        <v>629</v>
+        <v>414</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B341" t="s">
         <v>5</v>
       </c>
       <c r="C341" t="s">
-        <v>425</v>
+        <v>6</v>
       </c>
       <c r="D341" t="s">
-        <v>614</v>
+        <v>605</v>
       </c>
       <c r="E341" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="F341" s="5" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B342" t="s">
         <v>5</v>
       </c>
       <c r="C342" t="s">
-        <v>426</v>
+        <v>579</v>
       </c>
       <c r="D342" t="s">
-        <v>615</v>
+        <v>606</v>
       </c>
       <c r="E342" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="F342" s="5" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B343" t="s">
         <v>5</v>
       </c>
       <c r="C343" t="s">
-        <v>436</v>
+        <v>580</v>
       </c>
       <c r="D343" t="s">
-        <v>616</v>
+        <v>607</v>
       </c>
       <c r="E343" s="5" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B344" t="s">
         <v>5</v>
       </c>
       <c r="C344" t="s">
-        <v>437</v>
+        <v>581</v>
       </c>
       <c r="D344" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
       <c r="E344" s="5" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B345" t="s">
         <v>5</v>
       </c>
       <c r="C345" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="D345" t="s">
-        <v>618</v>
+        <v>609</v>
       </c>
       <c r="E345" s="5" t="s">
-        <v>633</v>
+        <v>628</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B346" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C346" t="s">
-        <v>6</v>
+        <v>421</v>
       </c>
       <c r="D346" t="s">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="E346" s="5" t="s">
-        <v>630</v>
+        <v>628</v>
+      </c>
+      <c r="F346" s="5" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B347" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C347" t="s">
-        <v>583</v>
+        <v>422</v>
       </c>
       <c r="D347" t="s">
-        <v>620</v>
+        <v>611</v>
       </c>
       <c r="E347" s="5" t="s">
-        <v>634</v>
+        <v>628</v>
+      </c>
+      <c r="F347" s="5" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B348" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C348" t="s">
-        <v>584</v>
+        <v>432</v>
       </c>
       <c r="D348" t="s">
-        <v>621</v>
+        <v>612</v>
       </c>
       <c r="E348" s="5" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B349" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C349" t="s">
-        <v>585</v>
+        <v>433</v>
       </c>
       <c r="D349" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="E349" s="5" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B350" t="s">
-        <v>588</v>
+        <v>5</v>
       </c>
       <c r="C350" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="D350" t="s">
-        <v>623</v>
+        <v>614</v>
       </c>
       <c r="E350" s="5" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B351" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C351" t="s">
-        <v>425</v>
+        <v>6</v>
       </c>
       <c r="D351" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="E351" s="5" t="s">
-        <v>634</v>
+        <v>626</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B352" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C352" t="s">
-        <v>426</v>
+        <v>579</v>
       </c>
       <c r="D352" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="E352" s="5" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B353" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C353" t="s">
-        <v>436</v>
+        <v>580</v>
       </c>
       <c r="D353" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="E353" s="5" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B354" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C354" t="s">
-        <v>437</v>
+        <v>581</v>
       </c>
       <c r="D354" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="E354" s="5" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B355" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C355" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="D355" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="E355" s="5" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="356" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E356" s="5"/>
+      <c r="A356" t="s">
+        <v>583</v>
+      </c>
+      <c r="B356" t="s">
+        <v>584</v>
+      </c>
+      <c r="C356" t="s">
+        <v>421</v>
+      </c>
+      <c r="D356" t="s">
+        <v>620</v>
+      </c>
+      <c r="E356" s="5" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="357" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E357" s="5"/>
+      <c r="A357" t="s">
+        <v>583</v>
+      </c>
+      <c r="B357" t="s">
+        <v>584</v>
+      </c>
+      <c r="C357" t="s">
+        <v>422</v>
+      </c>
+      <c r="D357" t="s">
+        <v>621</v>
+      </c>
+      <c r="E357" s="5" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A358" t="s">
+        <v>583</v>
+      </c>
+      <c r="B358" t="s">
+        <v>584</v>
+      </c>
+      <c r="C358" t="s">
+        <v>432</v>
+      </c>
+      <c r="D358" t="s">
+        <v>622</v>
+      </c>
+      <c r="E358" s="5" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A359" t="s">
+        <v>583</v>
+      </c>
+      <c r="B359" t="s">
+        <v>584</v>
+      </c>
+      <c r="C359" t="s">
+        <v>433</v>
+      </c>
+      <c r="D359" t="s">
+        <v>623</v>
+      </c>
+      <c r="E359" s="5" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A360" t="s">
+        <v>583</v>
+      </c>
+      <c r="B360" t="s">
+        <v>584</v>
+      </c>
+      <c r="C360" t="s">
+        <v>434</v>
+      </c>
+      <c r="D360" t="s">
+        <v>624</v>
+      </c>
+      <c r="E360" s="5" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E361" s="5"/>
+    </row>
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E362" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A313:L313"/>
+    <mergeCell ref="A320:L320"/>
+    <mergeCell ref="A231:L231"/>
+    <mergeCell ref="A245:L245"/>
+    <mergeCell ref="A262:L262"/>
+    <mergeCell ref="A276:L276"/>
+    <mergeCell ref="A285:L285"/>
     <mergeCell ref="A208:L208"/>
     <mergeCell ref="A178:L178"/>
     <mergeCell ref="A115:L115"/>
     <mergeCell ref="E1:H1"/>
     <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A308:L308"/>
-    <mergeCell ref="A315:L315"/>
-    <mergeCell ref="A231:L231"/>
-    <mergeCell ref="A240:L240"/>
-    <mergeCell ref="A257:L257"/>
-    <mergeCell ref="A271:L271"/>
-    <mergeCell ref="A280:L280"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>